<commit_message>
feat: switch email delivery to direct Gmail SMTP from muhammadtalhapro1 to hassantariq603 at 07:05 AM
</commit_message>
<xml_diff>
--- a/reports/2026-10-17/private_scholarships_report_2026-10-17.xlsx
+++ b/reports/2026-10-17/private_scholarships_report_2026-10-17.xlsx
@@ -2133,7 +2133,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-10-17 07:40 PKT</t>
+          <t>2026-10-17 07:59 PKT</t>
         </is>
       </c>
     </row>
@@ -2145,7 +2145,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>RUN-20261017-074058</t>
+          <t>RUN-20261017-075906</t>
         </is>
       </c>
     </row>

</xml_diff>